<commit_message>
fix(costs): formats % scénarios + 3 onglets Unit Economics, Funding, Setup
Scénarios :
- Marge brute % et EBITDA % maintenant formatés en pourcentage
  (F_MONO écrasait le number_format précédemment).

Nouveaux onglets :
- Unit Economics — LTV/CAC, payback CAC, magic number, lifetime,
  benchmarks SaaS B2B SMB. Now LTV/CAC 1.33 (early), Next 4.56,
  Later 9.19. Payback 15 → 7 → 5 mois.
- Funding schedule — trajectoire 18 mois (T+0 → T+17) avec courtiers,
  revenus, OpEx, levées (250k T+0 · 1.5M T+6), burn net, cash position
  cumulée. Démontre runway non interrompu jusqu'à Series A.
- Setup one-shot — coûts ponctuels lancement (incorporation, marques,
  DPIA Loi 25, pen-test, hardware cofondateurs, salon REM, etc.) avec
  sous-totaux par catégorie. Total ~78 k$ CAD.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/24_NextMove/klaris-cost-structure.xlsx
+++ b/24_NextMove/klaris-cost-structure.xlsx
@@ -13,6 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salaires &amp; talent" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scénarios" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Economics" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding schedule" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup one-shot" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +29,7 @@
     <numFmt numFmtId="165" formatCode="_-* #,##0.00 &quot;$&quot;_-;-* #,##0.00 &quot;$&quot;_-;_-* &quot;-&quot;?? &quot;$&quot;_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,6 +88,18 @@
       <b val="1"/>
       <color rgb="00C25A36"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="00C25A36"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="003D7A3A"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="14">
@@ -225,7 +240,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -394,6 +409,32 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5828,4 +5869,2094 @@
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Unit Economics — LTV / CAC / Payback</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Métriques par courtier acquis. Cible : LTV/CAC &gt; 3, payback &lt; 12 mois (benchmark SaaS B2B SMB).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Métrique</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Now (10c)</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Next (200c)</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Later (1000c)</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Formule / hypothèse</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>ARPU mensuel ($CAD)</t>
+        </is>
+      </c>
+      <c r="B5" s="44" t="n">
+        <v>100</v>
+      </c>
+      <c r="C5" s="44" t="n">
+        <v>125</v>
+      </c>
+      <c r="D5" s="44" t="n">
+        <v>150</v>
+      </c>
+      <c r="E5" s="21" t="inlineStr">
+        <is>
+          <t>Mix Solo / Agence / EN-CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Marge brute / courtier / mois</t>
+        </is>
+      </c>
+      <c r="B6" s="44">
+        <f>Scénarios!B6-'COGS variable'!B20</f>
+        <v/>
+      </c>
+      <c r="C6" s="44">
+        <f>Scénarios!C6-'COGS variable'!C20</f>
+        <v/>
+      </c>
+      <c r="D6" s="44">
+        <f>Scénarios!D6-'COGS variable'!D20</f>
+        <v/>
+      </c>
+      <c r="E6" s="21">
+        <f>'COGS variable'!B23 — lien dynamique</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Marge brute %</t>
+        </is>
+      </c>
+      <c r="B7" s="80">
+        <f>B6/B5</f>
+        <v/>
+      </c>
+      <c r="C7" s="80">
+        <f>C6/C5</f>
+        <v/>
+      </c>
+      <c r="D7" s="80">
+        <f>D6/D5</f>
+        <v/>
+      </c>
+      <c r="E7" s="21">
+        <f>'COGS variable'!B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Churn mensuel (% courtiers/mois)</t>
+        </is>
+      </c>
+      <c r="B8" s="80" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C8" s="80" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D8" s="80" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E8" s="21" t="inlineStr">
+        <is>
+          <t>5% Now (early pilots) → 2% Later (sticky agences)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Lifetime moyen (mois)</t>
+        </is>
+      </c>
+      <c r="B9" s="81">
+        <f>1/B8</f>
+        <v/>
+      </c>
+      <c r="C9" s="81">
+        <f>1/C8</f>
+        <v/>
+      </c>
+      <c r="D9" s="81">
+        <f>1/D8</f>
+        <v/>
+      </c>
+      <c r="E9" s="21">
+        <f> 1 / churn mensuel</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>LTV brute ($CAD)</t>
+        </is>
+      </c>
+      <c r="B10" s="20">
+        <f>B5*B9</f>
+        <v/>
+      </c>
+      <c r="C10" s="20">
+        <f>C5*C9</f>
+        <v/>
+      </c>
+      <c r="D10" s="20">
+        <f>D5*D9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f> ARPU × Lifetime</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="82" t="inlineStr">
+        <is>
+          <t>LTV marge brute ($CAD)</t>
+        </is>
+      </c>
+      <c r="B11" s="43">
+        <f>B6*B9</f>
+        <v/>
+      </c>
+      <c r="C11" s="43">
+        <f>C6*C9</f>
+        <v/>
+      </c>
+      <c r="D11" s="43">
+        <f>D6*D9</f>
+        <v/>
+      </c>
+      <c r="E11" s="21">
+        <f> Marge brute mensuelle × Lifetime</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="18" t="inlineStr"/>
+      <c r="B12" s="47" t="inlineStr"/>
+      <c r="C12" s="47" t="inlineStr"/>
+      <c r="D12" s="47" t="inlineStr"/>
+      <c r="E12" s="21" t="inlineStr"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Coût marketing mensuel ($CAD)</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="n">
+        <v>800</v>
+      </c>
+      <c r="C13" s="20" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <v>14500</v>
+      </c>
+      <c r="E13" s="21" t="inlineStr">
+        <is>
+          <t>Google + Meta + salons + freelance + Customer.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Coût sales mensuel ($CAD)</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C14" s="20" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D14" s="20" t="n">
+        <v>12500</v>
+      </c>
+      <c r="E14" s="21" t="inlineStr">
+        <is>
+          <t>Cofondateurs Now ; +rep Next ; +rep ON Later</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>CAC mensuel total ($CAD)</t>
+        </is>
+      </c>
+      <c r="B15" s="20">
+        <f>B13+B14</f>
+        <v/>
+      </c>
+      <c r="C15" s="20">
+        <f>C13+C14</f>
+        <v/>
+      </c>
+      <c r="D15" s="20">
+        <f>D13+D14</f>
+        <v/>
+      </c>
+      <c r="E15" s="21">
+        <f> Mkt + Sales</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Nouveaux courtiers acquis / mois</t>
+        </is>
+      </c>
+      <c r="B16" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="83" t="n">
+        <v>15</v>
+      </c>
+      <c r="D16" s="83" t="n">
+        <v>40</v>
+      </c>
+      <c r="E16" s="21" t="inlineStr">
+        <is>
+          <t>Taux d'acquisition net (gross − churn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="82" t="inlineStr">
+        <is>
+          <t>CAC par courtier ($CAD)</t>
+        </is>
+      </c>
+      <c r="B17" s="43">
+        <f>B15/B16</f>
+        <v/>
+      </c>
+      <c r="C17" s="43">
+        <f>C15/C16</f>
+        <v/>
+      </c>
+      <c r="D17" s="43">
+        <f>D15/D16</f>
+        <v/>
+      </c>
+      <c r="E17" s="21">
+        <f> CAC mensuel / acquisitions</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="18" t="inlineStr"/>
+      <c r="B18" s="47" t="inlineStr"/>
+      <c r="C18" s="47" t="inlineStr"/>
+      <c r="D18" s="47" t="inlineStr"/>
+      <c r="E18" s="21" t="inlineStr"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="82" t="inlineStr">
+        <is>
+          <t>LTV / CAC</t>
+        </is>
+      </c>
+      <c r="B19" s="84">
+        <f>B11/B17</f>
+        <v/>
+      </c>
+      <c r="C19" s="84">
+        <f>C11/C17</f>
+        <v/>
+      </c>
+      <c r="D19" s="84">
+        <f>D11/D17</f>
+        <v/>
+      </c>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
+          <t>Cible &gt; 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="82" t="inlineStr">
+        <is>
+          <t>Payback CAC (mois)</t>
+        </is>
+      </c>
+      <c r="B20" s="84">
+        <f>B17/B6</f>
+        <v/>
+      </c>
+      <c r="C20" s="84">
+        <f>C17/C6</f>
+        <v/>
+      </c>
+      <c r="D20" s="84">
+        <f>D17/D6</f>
+        <v/>
+      </c>
+      <c r="E20" s="21">
+        <f> CAC / Marge brute mensuelle</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Magic Number (efficience)</t>
+        </is>
+      </c>
+      <c r="B21" s="85">
+        <f>(B16*12*B5)/(B15*3)</f>
+        <v/>
+      </c>
+      <c r="C21" s="85">
+        <f>(C16*12*C5)/(C15*3)</f>
+        <v/>
+      </c>
+      <c r="D21" s="85">
+        <f>(D16*12*D5)/(D15*3)</f>
+        <v/>
+      </c>
+      <c r="E21" s="21">
+        <f> (ΔMRR × 4) / S&amp;M dépense trimestrielle. Cible &gt; 0,75</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Benchmarks SaaS B2B SMB (référence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>LTV / CAC sain</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>&gt; 3 (visé). &gt; 5 = scaling robuste.</t>
+        </is>
+      </c>
+      <c r="C25" s="47" t="n"/>
+      <c r="D25" s="47" t="n"/>
+      <c r="E25" s="47" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>Payback CAC</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>&lt; 12 mois early, &lt; 18 mois growth.</t>
+        </is>
+      </c>
+      <c r="C26" s="47" t="n"/>
+      <c r="D26" s="47" t="n"/>
+      <c r="E26" s="47" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Churn mensuel toléré</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>&lt; 3% PME, &lt; 1% entreprise.</t>
+        </is>
+      </c>
+      <c r="C27" s="47" t="n"/>
+      <c r="D27" s="47" t="n"/>
+      <c r="E27" s="47" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>Magic Number</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>&gt; 0,75 (efficient). &gt; 1 = double S&amp;M maintenant.</t>
+        </is>
+      </c>
+      <c r="C28" s="47" t="n"/>
+      <c r="D28" s="47" t="n"/>
+      <c r="E28" s="47" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B28:E28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Calendrier de financement — 18 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Encaissements (levées + revenus) vs décaissements mensuels. Cash position cumulée. Tous montants $CAD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Mois</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Courtiers</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Revenus</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>OpEx</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>Cash levé</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>Burn net</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>T+0 (Juin 2026)</t>
+        </is>
+      </c>
+      <c r="B5" s="86" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" s="20" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E5" s="20" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F5" s="20" t="n">
+        <v>250000</v>
+      </c>
+      <c r="G5" s="20" t="n">
+        <v>236000</v>
+      </c>
+      <c r="H5" s="21" t="inlineStr">
+        <is>
+          <t>Pré-amorçage closed · TestFlight launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>T+1</t>
+        </is>
+      </c>
+      <c r="B6" s="86" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="D6" s="20" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E6" s="20" t="n">
+        <v>16000</v>
+      </c>
+      <c r="F6" s="19" t="n"/>
+      <c r="G6" s="87" t="n">
+        <v>-14500</v>
+      </c>
+      <c r="H6" s="21" t="inlineStr">
+        <is>
+          <t>Captation OACIQ revue</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>T+2</t>
+        </is>
+      </c>
+      <c r="B7" s="86" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="D7" s="20" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E7" s="20" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F7" s="19" t="n"/>
+      <c r="G7" s="87" t="n">
+        <v>-15500</v>
+      </c>
+      <c r="H7" s="21" t="inlineStr">
+        <is>
+          <t>App Store live · acquisition courtier</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>T+3 (Sept)</t>
+        </is>
+      </c>
+      <c r="B8" s="86" t="inlineStr">
+        <is>
+          <t>Now→Next</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="D8" s="20" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>22000</v>
+      </c>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="87" t="n">
+        <v>-18000</v>
+      </c>
+      <c r="H8" s="21" t="inlineStr">
+        <is>
+          <t>Premier deal agence pilote</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>T+4</t>
+        </is>
+      </c>
+      <c r="B9" s="88" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>60</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <v>6300</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F9" s="19" t="n"/>
+      <c r="G9" s="87" t="n">
+        <v>-23700</v>
+      </c>
+      <c r="H9" s="21" t="inlineStr">
+        <is>
+          <t>Centris API négo + Notarius signé</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>T+5</t>
+        </is>
+      </c>
+      <c r="B10" s="88" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <v>9450</v>
+      </c>
+      <c r="E10" s="20" t="n">
+        <v>40000</v>
+      </c>
+      <c r="F10" s="19" t="n"/>
+      <c r="G10" s="87" t="n">
+        <v>-30550</v>
+      </c>
+      <c r="H10" s="21" t="inlineStr">
+        <is>
+          <t>Pré-Seed roadshow</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>T+6 (Déc 2026)</t>
+        </is>
+      </c>
+      <c r="B11" s="88" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>130</v>
+      </c>
+      <c r="D11" s="20" t="n">
+        <v>13650</v>
+      </c>
+      <c r="E11" s="20" t="n">
+        <v>55000</v>
+      </c>
+      <c r="F11" s="20" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="G11" s="20" t="n">
+        <v>1458650</v>
+      </c>
+      <c r="H11" s="21" t="inlineStr">
+        <is>
+          <t>Seed 1,5 M$ closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>T+7</t>
+        </is>
+      </c>
+      <c r="B12" s="88" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="n">
+        <v>165</v>
+      </c>
+      <c r="D12" s="20" t="n">
+        <v>17325</v>
+      </c>
+      <c r="E12" s="20" t="n">
+        <v>65000</v>
+      </c>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="87" t="n">
+        <v>-47675</v>
+      </c>
+      <c r="H12" s="21" t="inlineStr">
+        <is>
+          <t>Recrutements dev + sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>T+8 (Févr 2027)</t>
+        </is>
+      </c>
+      <c r="B13" s="88" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <v>23000</v>
+      </c>
+      <c r="E13" s="20" t="n">
+        <v>75000</v>
+      </c>
+      <c r="F13" s="19" t="n"/>
+      <c r="G13" s="87" t="n">
+        <v>-52000</v>
+      </c>
+      <c r="H13" s="21" t="inlineStr">
+        <is>
+          <t>Cible Next atteinte · 200 courtiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>T+9</t>
+        </is>
+      </c>
+      <c r="B14" s="88" t="inlineStr">
+        <is>
+          <t>Next→Later</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="n">
+        <v>250</v>
+      </c>
+      <c r="D14" s="20" t="n">
+        <v>28750</v>
+      </c>
+      <c r="E14" s="20" t="n">
+        <v>85000</v>
+      </c>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="87" t="n">
+        <v>-56250</v>
+      </c>
+      <c r="H14" s="21" t="inlineStr">
+        <is>
+          <t>Toronto launch préparé</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>T+10 (Avr 2027)</t>
+        </is>
+      </c>
+      <c r="B15" s="89" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="n">
+        <v>320</v>
+      </c>
+      <c r="D15" s="20" t="n">
+        <v>36800</v>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="87" t="n">
+        <v>-63200</v>
+      </c>
+      <c r="H15" s="21" t="inlineStr">
+        <is>
+          <t>Toronto + Ottawa go-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>T+11</t>
+        </is>
+      </c>
+      <c r="B16" s="89" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="n">
+        <v>400</v>
+      </c>
+      <c r="D16" s="20" t="n">
+        <v>46000</v>
+      </c>
+      <c r="E16" s="20" t="n">
+        <v>110000</v>
+      </c>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="87" t="n">
+        <v>-64000</v>
+      </c>
+      <c r="H16" s="21" t="inlineStr">
+        <is>
+          <t>Mid-market 1ʳᵉ vente 50+ courtiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>T+12</t>
+        </is>
+      </c>
+      <c r="B17" s="89" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="n">
+        <v>500</v>
+      </c>
+      <c r="D17" s="20" t="n">
+        <v>65000</v>
+      </c>
+      <c r="E17" s="20" t="n">
+        <v>115000</v>
+      </c>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="87" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="H17" s="21" t="inlineStr">
+        <is>
+          <t>Cible Later début · 500 courtiers · MRR 60k</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>T+13 (Juil 2027)</t>
+        </is>
+      </c>
+      <c r="B18" s="89" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>600</v>
+      </c>
+      <c r="D18" s="20" t="n">
+        <v>78000</v>
+      </c>
+      <c r="E18" s="20" t="n">
+        <v>125000</v>
+      </c>
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="87" t="n">
+        <v>-47000</v>
+      </c>
+      <c r="H18" s="21" t="inlineStr">
+        <is>
+          <t>Sprint 8 GA — rédac offres OACIQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>T+14</t>
+        </is>
+      </c>
+      <c r="B19" s="89" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="n">
+        <v>700</v>
+      </c>
+      <c r="D19" s="20" t="n">
+        <v>91000</v>
+      </c>
+      <c r="E19" s="20" t="n">
+        <v>130000</v>
+      </c>
+      <c r="F19" s="19" t="n"/>
+      <c r="G19" s="87" t="n">
+        <v>-39000</v>
+      </c>
+      <c r="H19" s="21" t="inlineStr">
+        <is>
+          <t>Notarius + DocuSign GA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>T+15</t>
+        </is>
+      </c>
+      <c r="B20" s="89" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="n">
+        <v>800</v>
+      </c>
+      <c r="D20" s="20" t="n">
+        <v>116000</v>
+      </c>
+      <c r="E20" s="20" t="n">
+        <v>135000</v>
+      </c>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="87" t="n">
+        <v>-19000</v>
+      </c>
+      <c r="H20" s="21" t="inlineStr">
+        <is>
+          <t>Marge &gt; 75% · platform API beta</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>T+16 (Oct 2027)</t>
+        </is>
+      </c>
+      <c r="B21" s="89" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="n">
+        <v>900</v>
+      </c>
+      <c r="D21" s="20" t="n">
+        <v>130500</v>
+      </c>
+      <c r="E21" s="20" t="n">
+        <v>140000</v>
+      </c>
+      <c r="F21" s="19" t="n"/>
+      <c r="G21" s="87" t="n">
+        <v>-9500</v>
+      </c>
+      <c r="H21" s="21" t="inlineStr">
+        <is>
+          <t>Conversations Series A (term sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>T+17 (Nov 2027)</t>
+        </is>
+      </c>
+      <c r="B22" s="89" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D22" s="20" t="n">
+        <v>145000</v>
+      </c>
+      <c r="E22" s="20" t="n">
+        <v>140000</v>
+      </c>
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="90" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H22" s="21" t="inlineStr">
+        <is>
+          <t>Cible Later atteinte · ARR 1,5M$</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="42" t="inlineStr">
+        <is>
+          <t>Cash position cumulée (fin de période)</t>
+        </is>
+      </c>
+      <c r="B24" s="41" t="n"/>
+      <c r="C24" s="41" t="n"/>
+      <c r="D24" s="41" t="n"/>
+      <c r="E24" s="41" t="n"/>
+      <c r="F24" s="41" t="n"/>
+      <c r="G24" s="41" t="n"/>
+      <c r="H24" s="41" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Cash début T+0</t>
+        </is>
+      </c>
+      <c r="B25" s="47" t="n"/>
+      <c r="C25" s="47" t="n"/>
+      <c r="D25" s="47" t="n"/>
+      <c r="E25" s="47" t="n"/>
+      <c r="F25" s="47" t="n"/>
+      <c r="G25" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="47" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>T+0 (Juin 2026)</t>
+        </is>
+      </c>
+      <c r="B26" s="47" t="n"/>
+      <c r="C26" s="47" t="n"/>
+      <c r="D26" s="47" t="n"/>
+      <c r="E26" s="47" t="n"/>
+      <c r="F26" s="47" t="n"/>
+      <c r="G26" s="20">
+        <f>G25+G5</f>
+        <v/>
+      </c>
+      <c r="H26" s="47" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>T+1</t>
+        </is>
+      </c>
+      <c r="B27" s="47" t="n"/>
+      <c r="C27" s="47" t="n"/>
+      <c r="D27" s="47" t="n"/>
+      <c r="E27" s="47" t="n"/>
+      <c r="F27" s="47" t="n"/>
+      <c r="G27" s="20">
+        <f>G26+G6</f>
+        <v/>
+      </c>
+      <c r="H27" s="47" t="n"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>T+2</t>
+        </is>
+      </c>
+      <c r="B28" s="47" t="n"/>
+      <c r="C28" s="47" t="n"/>
+      <c r="D28" s="47" t="n"/>
+      <c r="E28" s="47" t="n"/>
+      <c r="F28" s="47" t="n"/>
+      <c r="G28" s="20">
+        <f>G27+G7</f>
+        <v/>
+      </c>
+      <c r="H28" s="47" t="n"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>T+3 (Sept)</t>
+        </is>
+      </c>
+      <c r="B29" s="47" t="n"/>
+      <c r="C29" s="47" t="n"/>
+      <c r="D29" s="47" t="n"/>
+      <c r="E29" s="47" t="n"/>
+      <c r="F29" s="47" t="n"/>
+      <c r="G29" s="20">
+        <f>G28+G8</f>
+        <v/>
+      </c>
+      <c r="H29" s="47" t="n"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>T+4</t>
+        </is>
+      </c>
+      <c r="B30" s="47" t="n"/>
+      <c r="C30" s="47" t="n"/>
+      <c r="D30" s="47" t="n"/>
+      <c r="E30" s="47" t="n"/>
+      <c r="F30" s="47" t="n"/>
+      <c r="G30" s="20">
+        <f>G29+G9</f>
+        <v/>
+      </c>
+      <c r="H30" s="47" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>T+5</t>
+        </is>
+      </c>
+      <c r="B31" s="47" t="n"/>
+      <c r="C31" s="47" t="n"/>
+      <c r="D31" s="47" t="n"/>
+      <c r="E31" s="47" t="n"/>
+      <c r="F31" s="47" t="n"/>
+      <c r="G31" s="20">
+        <f>G30+G10</f>
+        <v/>
+      </c>
+      <c r="H31" s="47" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>T+6 (Déc 2026)</t>
+        </is>
+      </c>
+      <c r="B32" s="47" t="n"/>
+      <c r="C32" s="47" t="n"/>
+      <c r="D32" s="47" t="n"/>
+      <c r="E32" s="47" t="n"/>
+      <c r="F32" s="47" t="n"/>
+      <c r="G32" s="20">
+        <f>G31+G11</f>
+        <v/>
+      </c>
+      <c r="H32" s="47" t="n"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="18" t="inlineStr">
+        <is>
+          <t>T+7</t>
+        </is>
+      </c>
+      <c r="B33" s="47" t="n"/>
+      <c r="C33" s="47" t="n"/>
+      <c r="D33" s="47" t="n"/>
+      <c r="E33" s="47" t="n"/>
+      <c r="F33" s="47" t="n"/>
+      <c r="G33" s="20">
+        <f>G32+G12</f>
+        <v/>
+      </c>
+      <c r="H33" s="47" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>T+8 (Févr 2027)</t>
+        </is>
+      </c>
+      <c r="B34" s="47" t="n"/>
+      <c r="C34" s="47" t="n"/>
+      <c r="D34" s="47" t="n"/>
+      <c r="E34" s="47" t="n"/>
+      <c r="F34" s="47" t="n"/>
+      <c r="G34" s="20">
+        <f>G33+G13</f>
+        <v/>
+      </c>
+      <c r="H34" s="47" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="18" t="inlineStr">
+        <is>
+          <t>T+9</t>
+        </is>
+      </c>
+      <c r="B35" s="47" t="n"/>
+      <c r="C35" s="47" t="n"/>
+      <c r="D35" s="47" t="n"/>
+      <c r="E35" s="47" t="n"/>
+      <c r="F35" s="47" t="n"/>
+      <c r="G35" s="20">
+        <f>G34+G14</f>
+        <v/>
+      </c>
+      <c r="H35" s="47" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="18" t="inlineStr">
+        <is>
+          <t>T+10 (Avr 2027)</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="n"/>
+      <c r="C36" s="47" t="n"/>
+      <c r="D36" s="47" t="n"/>
+      <c r="E36" s="47" t="n"/>
+      <c r="F36" s="47" t="n"/>
+      <c r="G36" s="20">
+        <f>G35+G15</f>
+        <v/>
+      </c>
+      <c r="H36" s="47" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="18" t="inlineStr">
+        <is>
+          <t>T+11</t>
+        </is>
+      </c>
+      <c r="B37" s="47" t="n"/>
+      <c r="C37" s="47" t="n"/>
+      <c r="D37" s="47" t="n"/>
+      <c r="E37" s="47" t="n"/>
+      <c r="F37" s="47" t="n"/>
+      <c r="G37" s="20">
+        <f>G36+G16</f>
+        <v/>
+      </c>
+      <c r="H37" s="47" t="n"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="18" t="inlineStr">
+        <is>
+          <t>T+12</t>
+        </is>
+      </c>
+      <c r="B38" s="47" t="n"/>
+      <c r="C38" s="47" t="n"/>
+      <c r="D38" s="47" t="n"/>
+      <c r="E38" s="47" t="n"/>
+      <c r="F38" s="47" t="n"/>
+      <c r="G38" s="20">
+        <f>G37+G17</f>
+        <v/>
+      </c>
+      <c r="H38" s="47" t="n"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="18" t="inlineStr">
+        <is>
+          <t>T+13 (Juil 2027)</t>
+        </is>
+      </c>
+      <c r="B39" s="47" t="n"/>
+      <c r="C39" s="47" t="n"/>
+      <c r="D39" s="47" t="n"/>
+      <c r="E39" s="47" t="n"/>
+      <c r="F39" s="47" t="n"/>
+      <c r="G39" s="20">
+        <f>G38+G18</f>
+        <v/>
+      </c>
+      <c r="H39" s="47" t="n"/>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="18" t="inlineStr">
+        <is>
+          <t>T+14</t>
+        </is>
+      </c>
+      <c r="B40" s="47" t="n"/>
+      <c r="C40" s="47" t="n"/>
+      <c r="D40" s="47" t="n"/>
+      <c r="E40" s="47" t="n"/>
+      <c r="F40" s="47" t="n"/>
+      <c r="G40" s="20">
+        <f>G39+G19</f>
+        <v/>
+      </c>
+      <c r="H40" s="47" t="n"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="18" t="inlineStr">
+        <is>
+          <t>T+15</t>
+        </is>
+      </c>
+      <c r="B41" s="47" t="n"/>
+      <c r="C41" s="47" t="n"/>
+      <c r="D41" s="47" t="n"/>
+      <c r="E41" s="47" t="n"/>
+      <c r="F41" s="47" t="n"/>
+      <c r="G41" s="20">
+        <f>G40+G20</f>
+        <v/>
+      </c>
+      <c r="H41" s="47" t="n"/>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="18" t="inlineStr">
+        <is>
+          <t>T+16 (Oct 2027)</t>
+        </is>
+      </c>
+      <c r="B42" s="47" t="n"/>
+      <c r="C42" s="47" t="n"/>
+      <c r="D42" s="47" t="n"/>
+      <c r="E42" s="47" t="n"/>
+      <c r="F42" s="47" t="n"/>
+      <c r="G42" s="20">
+        <f>G41+G21</f>
+        <v/>
+      </c>
+      <c r="H42" s="47" t="n"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="18" t="inlineStr">
+        <is>
+          <t>T+17 (Nov 2027)</t>
+        </is>
+      </c>
+      <c r="B43" s="47" t="n"/>
+      <c r="C43" s="47" t="n"/>
+      <c r="D43" s="47" t="n"/>
+      <c r="E43" s="47" t="n"/>
+      <c r="F43" s="47" t="n"/>
+      <c r="G43" s="20">
+        <f>G42+G22</f>
+        <v/>
+      </c>
+      <c r="H43" s="47" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="42" t="inlineStr">
+        <is>
+          <t>Total levée 18 mois</t>
+        </is>
+      </c>
+      <c r="B45" s="41" t="n"/>
+      <c r="C45" s="41" t="n"/>
+      <c r="D45" s="41" t="n"/>
+      <c r="E45" s="41" t="n"/>
+      <c r="F45" s="43">
+        <f>SUM(F5:F22)</f>
+        <v/>
+      </c>
+      <c r="G45" s="41" t="n"/>
+      <c r="H45" s="91" t="inlineStr">
+        <is>
+          <t>Pré-amorçage 250 k$ + Seed 1,5 M$ = 1,75 M$</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Coûts ponctuels de lancement (one-shot, hors mensuel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Investissements non récurrents — incorporation, propriété intellectuelle, hardware, dépôts initiaux.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Poste</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Catégorie</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Montant $CAD</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Incorporation fédérale + QC</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Légal</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="n">
+        <v>500</v>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>Frais gouvernementaux Industrie Canada + RBQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Convention d'actionnaires</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Légal</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>Vesting cofondateurs, drag/tag along, ROFR</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Marque déposée 'Klaris' CA + US</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>OPIC Canada + USPTO USA (2 classes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Marque 'Next Move'</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>OPIC Canada classe 9 + 42</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Politique conf. + DPIA Loi 25 init.</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>Rédaction initiale par DPO externe</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Adhésion OACIQ (revue conformité)</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>Audit initial + lettre absence d'objection</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Pen-test initial</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
+        <is>
+          <t>Pré-Seed — boîte spécialisée Mtl</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Audit sécurité Supabase config</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>Revue RLS + secrets management</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>4× MacBook Pro M4 (cofondateurs)</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="n">
+        <v>14000</v>
+      </c>
+      <c r="D13" s="21" t="inlineStr">
+        <is>
+          <t>16'' M4 Pro 24 Go / 1 To</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>3× écrans 4K 27''</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>Workstation cofondateurs tech</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Mobiliers + ergonomie</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D15" s="21" t="inlineStr">
+        <is>
+          <t>Chaises, bureaux, casques</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>4× iPhone 16 Pro (tests + démos)</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D16" s="21" t="inlineStr">
+        <is>
+          <t>Test app + démos courtiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>2× Apple Watch Series 10</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="n">
+        <v>1400</v>
+      </c>
+      <c r="D17" s="21" t="inlineStr">
+        <is>
+          <t>Test companion app</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>iPad Pro M4 (démos terrain)</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>Présentations courtiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>Site klaris.app + landing</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D19" s="21" t="inlineStr">
+        <is>
+          <t>Design + dev custom Next.js (déjà partiellement livré)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Pitch deck + identité visuelle</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D20" s="21" t="inlineStr">
+        <is>
+          <t>Direction artistique terracotta + logo</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Captation vidéo démo + témoignages</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D21" s="21" t="inlineStr">
+        <is>
+          <t>Vidéaste + montage 3 vidéos (60s, 30s, 15s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Pilote terrain — incentives</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Acquisition</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>Cartes cadeaux pilotes (Joanel + 9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Salon REM 2026 (stand + frais)</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>Acquisition</t>
+        </is>
+      </c>
+      <c r="C23" s="20" t="n">
+        <v>5500</v>
+      </c>
+      <c r="D23" s="21" t="inlineStr">
+        <is>
+          <t>Présence salon courtiers QC</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Comptable — bouclage initial</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D24" s="21" t="inlineStr">
+        <is>
+          <t>Bilan ouverture + structures fiscales</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Provision contingence</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>Réserve</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D25" s="21" t="inlineStr">
+        <is>
+          <t>Imprévus (5–10% du total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="42" t="inlineStr">
+        <is>
+          <t>TOTAL SETUP ONE-SHOT</t>
+        </is>
+      </c>
+      <c r="B27" s="41" t="n"/>
+      <c r="C27" s="43">
+        <f>SUM(C5:C25)</f>
+        <v/>
+      </c>
+      <c r="D27" s="41" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Sous-totaux par catégorie</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Légal</t>
+        </is>
+      </c>
+      <c r="B30" s="47" t="n"/>
+      <c r="C30" s="20">
+        <f>SUMIF(B5:B25,"Légal",C5:C25)</f>
+        <v/>
+      </c>
+      <c r="D30" s="47" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B31" s="47" t="n"/>
+      <c r="C31" s="20">
+        <f>SUMIF(B5:B25,"PI",C5:C25)</f>
+        <v/>
+      </c>
+      <c r="D31" s="47" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="B32" s="47" t="n"/>
+      <c r="C32" s="20">
+        <f>SUMIF(B5:B25,"Conformité",C5:C25)</f>
+        <v/>
+      </c>
+      <c r="D32" s="47" t="n"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="B33" s="47" t="n"/>
+      <c r="C33" s="20">
+        <f>SUMIF(B5:B25,"Sécurité",C5:C25)</f>
+        <v/>
+      </c>
+      <c r="D33" s="47" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="B34" s="47" t="n"/>
+      <c r="C34" s="20">
+        <f>SUMIF(B5:B25,"Hardware",C5:C25)</f>
+        <v/>
+      </c>
+      <c r="D34" s="47" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B35" s="47" t="n"/>
+      <c r="C35" s="20">
+        <f>SUMIF(B5:B25,"Marketing",C5:C25)</f>
+        <v/>
+      </c>
+      <c r="D35" s="47" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>Acquisition</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="n"/>
+      <c r="C36" s="20">
+        <f>SUMIF(B5:B25,"Acquisition",C5:C25)</f>
+        <v/>
+      </c>
+      <c r="D36" s="47" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="B37" s="47" t="n"/>
+      <c r="C37" s="20">
+        <f>SUMIF(B5:B25,"Admin",C5:C25)</f>
+        <v/>
+      </c>
+      <c r="D37" s="47" t="n"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>Réserve</t>
+        </is>
+      </c>
+      <c r="B38" s="47" t="n"/>
+      <c r="C38" s="20">
+        <f>SUMIF(B5:B25,"Réserve",C5:C25)</f>
+        <v/>
+      </c>
+      <c r="D38" s="47" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(confidence): méthodologie scoring % roadmap + onglet xlsx
Nouveau doc klaris-confidence-methodology.md :
- Formule : Confidence = (D×0,25 + C×0,25 + X×0,15 + M×0,25 + R×0,10) / 5 × 100
- 5 facteurs (Discovery · Capacity · Dependencies · Market · Regulatory)
  notés 0–5 avec grilles détaillées par facteur.
- Plafond 90% (règle prr), plancher 15%.
- 'Discount prudence' (petit n / externe / marché nouveau) : asymétrie
  volontaire — on baisse jamais on ne monte.
- Application à 20+ thèmes : Calculée vs Affichée + justification.
- Cadence revue (hebdo D/C, mensuelle X/M/R, trimestrielle full re-scoring).
- Limites + section investisseurs (comment auditer un score).

Onglet xlsx Confidence scoring :
- 22 thèmes scorés D/C/X/M/R avec formules vivantes (édite, recalcule).
- Color scale rouge → ambre → vert sur colonne Affichée.
- Grille de notation 0-5 par facteur en référence intégrée.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/24_NextMove/klaris-cost-structure.xlsx
+++ b/24_NextMove/klaris-cost-structure.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Economics" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding schedule" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup one-shot" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confidence scoring" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,12 +25,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="_-* #,##0 &quot;$&quot;_-;-* #,##0 &quot;$&quot;_-;_-* &quot;-&quot;?? &quot;$&quot;_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00 &quot;$&quot;_-;-* #,##0.00 &quot;$&quot;_-;_-* &quot;-&quot;?? &quot;$&quot;_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="+0%;-0%;0%"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -99,6 +101,11 @@
       <name val="Consolas"/>
       <b val="1"/>
       <color rgb="003D7A3A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="00C25A36"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -240,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -435,6 +442,42 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1105,6 +1148,1400 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Méthodologie de scoring des % de confiance — roadmap</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Formule : Confidence = (D × 0,25 + C × 0,25 + X × 0,15 + M × 0,25 + R × 0,10) / 5 × 100. Plafond 90% (règle prr). 'Discount' = ajustement prudence appliqué.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="92" t="inlineStr">
+        <is>
+          <t>Pondérations</t>
+        </is>
+      </c>
+      <c r="B3" s="93" t="n"/>
+      <c r="C3" s="92" t="inlineStr">
+        <is>
+          <t>D 25%</t>
+        </is>
+      </c>
+      <c r="D3" s="92" t="inlineStr">
+        <is>
+          <t>C 25%</t>
+        </is>
+      </c>
+      <c r="E3" s="92" t="inlineStr">
+        <is>
+          <t>X 15%</t>
+        </is>
+      </c>
+      <c r="F3" s="92" t="inlineStr">
+        <is>
+          <t>M 25%</t>
+        </is>
+      </c>
+      <c r="G3" s="92" t="inlineStr">
+        <is>
+          <t>R 10%</t>
+        </is>
+      </c>
+      <c r="H3" s="93" t="n"/>
+      <c r="I3" s="93" t="n"/>
+      <c r="J3" s="93" t="n"/>
+      <c r="K3" s="93" t="n"/>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Thème</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Horizon</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>Calculée</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>Discount</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Affichée</t>
+        </is>
+      </c>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="94" t="inlineStr">
+        <is>
+          <t>Pilotes convertissent leurs leads sans admin manuel</t>
+        </is>
+      </c>
+      <c r="B6" s="95" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="C6" s="96" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="96" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="96" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" s="97">
+        <f>MIN(0.9, (C6*0.25 + D6*0.25 + E6*0.15 + F6*0.25 + G6*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I6" s="98" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="J6" s="99">
+        <f>MAX(0.15, H6 + I6)</f>
+        <v/>
+      </c>
+      <c r="K6" s="21" t="inlineStr">
+        <is>
+          <t>Plafond 90% appliqué ; discount -10 pour pilote unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="94" t="inlineStr">
+        <is>
+          <t>OACIQ reconnaît Klaris conforme par défaut</t>
+        </is>
+      </c>
+      <c r="B7" s="95" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="C7" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="97">
+        <f>MIN(0.9, (C7*0.25 + D7*0.25 + E7*0.15 + F7*0.25 + G7*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I7" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="99">
+        <f>MAX(0.15, H7 + I7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="21" t="inlineStr">
+        <is>
+          <t>Démarche en cours, dépend régulateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="94" t="inlineStr">
+        <is>
+          <t>Pilotes restent payants au-delà de 90 jours</t>
+        </is>
+      </c>
+      <c r="B8" s="95" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="C8" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" s="97">
+        <f>MIN(0.9, (C8*0.25 + D8*0.25 + E8*0.15 + F8*0.25 + G8*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I8" s="98" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="J8" s="99">
+        <f>MAX(0.15, H8 + I8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="21" t="inlineStr">
+        <is>
+          <t>Données &lt; 90 j — incertitude rétention</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="94" t="inlineStr">
+        <is>
+          <t>Investisseurs pré-amorçage : signal commercial clair</t>
+        </is>
+      </c>
+      <c r="B9" s="95" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="C9" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="97">
+        <f>MIN(0.9, (C9*0.25 + D9*0.25 + E9*0.15 + F9*0.25 + G9*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I9" s="98" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="J9" s="99">
+        <f>MAX(0.15, H9 + I9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="21" t="inlineStr">
+        <is>
+          <t>Externe — moins maîtrisé</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="94" t="inlineStr">
+        <is>
+          <t>Agences pilotent équipe depuis un seul dashboard</t>
+        </is>
+      </c>
+      <c r="B10" s="101" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="C10" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="H10" s="97">
+        <f>MIN(0.9, (C10*0.25 + D10*0.25 + E10*0.15 + F10*0.25 + G10*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I10" s="98" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="J10" s="99">
+        <f>MAX(0.15, H10 + I10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="21" t="inlineStr">
+        <is>
+          <t>Dashboard scaffold prêt, RBAC à durcir</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="94" t="inlineStr">
+        <is>
+          <t>Fiches Centris sans re-saisie</t>
+        </is>
+      </c>
+      <c r="B11" s="101" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="C11" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="96" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" s="97">
+        <f>MIN(0.9, (C11*0.25 + D11*0.25 + E11*0.15 + F11*0.25 + G11*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I11" s="98" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="J11" s="99">
+        <f>MAX(0.15, H11 + I11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="21" t="inlineStr">
+        <is>
+          <t>X faible : API Centris non publique</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="94" t="inlineStr">
+        <is>
+          <t>Offre passe du chat à e-signature en un flux</t>
+        </is>
+      </c>
+      <c r="B12" s="101" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="C12" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" s="97">
+        <f>MIN(0.9, (C12*0.25 + D12*0.25 + E12*0.15 + F12*0.25 + G12*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I12" s="98" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="J12" s="99">
+        <f>MAX(0.15, H12 + I12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="21" t="inlineStr">
+        <is>
+          <t>Intégration Notarius non encore validée</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="94" t="inlineStr">
+        <is>
+          <t>VCs Seed : thèse Canada défendable</t>
+        </is>
+      </c>
+      <c r="B13" s="101" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="C13" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" s="97">
+        <f>MIN(0.9, (C13*0.25 + D13*0.25 + E13*0.15 + F13*0.25 + G13*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I13" s="98" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="J13" s="99">
+        <f>MAX(0.15, H13 + I13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="21" t="inlineStr">
+        <is>
+          <t>Externe + dépend traction Next</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="94" t="inlineStr">
+        <is>
+          <t>Klaris parle au marché anglo-canadien</t>
+        </is>
+      </c>
+      <c r="B14" s="102" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C14" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" s="97">
+        <f>MIN(0.9, (C14*0.25 + D14*0.25 + E14*0.15 + F14*0.25 + G14*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I14" s="98" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="J14" s="99">
+        <f>MAX(0.15, H14 + I14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="21" t="inlineStr">
+        <is>
+          <t>Marché nouveau, M revu prudent</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="94" t="inlineStr">
+        <is>
+          <t>Garder relation client post-closing</t>
+        </is>
+      </c>
+      <c r="B15" s="102" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C15" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" s="97">
+        <f>MIN(0.9, (C15*0.25 + D15*0.25 + E15*0.15 + F15*0.25 + G15*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I15" s="98" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="J15" s="99">
+        <f>MAX(0.15, H15 + I15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="21" t="inlineStr">
+        <is>
+          <t>Priorisation incertaine vs autres thèmes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="94" t="inlineStr">
+        <is>
+          <t>Partenaires intègrent Klaris (CRMs, prêteurs)</t>
+        </is>
+      </c>
+      <c r="B16" s="102" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C16" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="H16" s="97">
+        <f>MIN(0.9, (C16*0.25 + D16*0.25 + E16*0.15 + F16*0.25 + G16*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I16" s="98" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="J16" s="99">
+        <f>MAX(0.15, H16 + I16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="21" t="inlineStr">
+        <is>
+          <t>API publique encore à designer</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="94" t="inlineStr">
+        <is>
+          <t>Marketplace prospects qualifiés</t>
+        </is>
+      </c>
+      <c r="B17" s="102" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C17" s="96" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="96" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="96" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="97">
+        <f>MIN(0.9, (C17*0.25 + D17*0.25 + E17*0.15 + F17*0.25 + G17*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I17" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="99">
+        <f>MAX(0.15, H17 + I17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="21" t="inlineStr">
+        <is>
+          <t>Hypothèse marché non testée</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="94" t="inlineStr">
+        <is>
+          <t>Audit log PII complet (Loi 25)</t>
+        </is>
+      </c>
+      <c r="B18" s="95" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="C18" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="96" t="n">
+        <v>5</v>
+      </c>
+      <c r="E18" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="F18" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" s="96" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" s="97">
+        <f>MIN(0.9, (C18*0.25 + D18*0.25 + E18*0.15 + F18*0.25 + G18*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I18" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="99">
+        <f>MAX(0.15, H18 + I18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="21" t="inlineStr">
+        <is>
+          <t>Migration prête, juste à déployer</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="94" t="inlineStr">
+        <is>
+          <t>Backups + DR Supabase (PITR + drill mensuel)</t>
+        </is>
+      </c>
+      <c r="B19" s="95" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="C19" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="96" t="n">
+        <v>5</v>
+      </c>
+      <c r="E19" s="96" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="G19" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="H19" s="97">
+        <f>MIN(0.9, (C19*0.25 + D19*0.25 + E19*0.15 + F19*0.25 + G19*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I19" s="98" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="J19" s="99">
+        <f>MAX(0.15, H19 + I19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="21" t="inlineStr">
+        <is>
+          <t>Drill à institutionnaliser</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="94" t="inlineStr">
+        <is>
+          <t>Eval suite IA — ton QC + accuracy qualification</t>
+        </is>
+      </c>
+      <c r="B20" s="95" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="C20" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" s="96" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="G20" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="H20" s="97">
+        <f>MIN(0.9, (C20*0.25 + D20*0.25 + E20*0.15 + F20*0.25 + G20*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I20" s="98" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="J20" s="99">
+        <f>MAX(0.15, H20 + I20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="21" t="inlineStr">
+        <is>
+          <t>Dataset eval à étoffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="94" t="inlineStr">
+        <is>
+          <t>RAG V1 — base de connaissances agence</t>
+        </is>
+      </c>
+      <c r="B21" s="95" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="C21" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="H21" s="97">
+        <f>MIN(0.9, (C21*0.25 + D21*0.25 + E21*0.15 + F21*0.25 + G21*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I21" s="98" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="J21" s="99">
+        <f>MAX(0.15, H21 + I21)</f>
+        <v/>
+      </c>
+      <c r="K21" s="21" t="inlineStr">
+        <is>
+          <t>pgvector OK, chunking à valider</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="94" t="inlineStr">
+        <is>
+          <t>RAG V2 — multi-source hybrid (BM25 + rerank)</t>
+        </is>
+      </c>
+      <c r="B22" s="101" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="C22" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="F22" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="H22" s="97">
+        <f>MIN(0.9, (C22*0.25 + D22*0.25 + E22*0.15 + F22*0.25 + G22*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I22" s="98" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="J22" s="99">
+        <f>MAX(0.15, H22 + I22)</f>
+        <v/>
+      </c>
+      <c r="K22" s="21" t="inlineStr">
+        <is>
+          <t>Voyage AI à benchmark vs OpenAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="94" t="inlineStr">
+        <is>
+          <t>RAG V3 — agentique (Claude tool-calls)</t>
+        </is>
+      </c>
+      <c r="B23" s="101" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="C23" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" s="97">
+        <f>MIN(0.9, (C23*0.25 + D23*0.25 + E23*0.15 + F23*0.25 + G23*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I23" s="98" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="J23" s="99">
+        <f>MAX(0.15, H23 + I23)</f>
+        <v/>
+      </c>
+      <c r="K23" s="21" t="inlineStr">
+        <is>
+          <t>Discovery requise</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="94" t="inlineStr">
+        <is>
+          <t>Mistral fallback opérationnel</t>
+        </is>
+      </c>
+      <c r="B24" s="101" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="C24" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="F24" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="H24" s="97">
+        <f>MIN(0.9, (C24*0.25 + D24*0.25 + E24*0.15 + F24*0.25 + G24*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I24" s="98" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="J24" s="99">
+        <f>MAX(0.15, H24 + I24)</f>
+        <v/>
+      </c>
+      <c r="K24" s="21" t="inlineStr">
+        <is>
+          <t>Plan B Anthropic — pas critique court terme</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="94" t="inlineStr">
+        <is>
+          <t>API publique v1 (OAuth, rate-limit, docs)</t>
+        </is>
+      </c>
+      <c r="B25" s="102" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C25" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="H25" s="97">
+        <f>MIN(0.9, (C25*0.25 + D25*0.25 + E25*0.15 + F25*0.25 + G25*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I25" s="98" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="J25" s="99">
+        <f>MAX(0.15, H25 + I25)</f>
+        <v/>
+      </c>
+      <c r="K25" s="21" t="inlineStr">
+        <is>
+          <t>Designer interface partenaires</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="94" t="inlineStr">
+        <is>
+          <t>Migrer n8n → service Python dédié</t>
+        </is>
+      </c>
+      <c r="B26" s="102" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C26" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="E26" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="F26" s="96" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="H26" s="97">
+        <f>MIN(0.9, (C26*0.25 + D26*0.25 + E26*0.15 + F26*0.25 + G26*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I26" s="98" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="J26" s="99">
+        <f>MAX(0.15, H26 + I26)</f>
+        <v/>
+      </c>
+      <c r="K26" s="21" t="inlineStr">
+        <is>
+          <t>Quand volume justifie</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="94" t="inlineStr">
+        <is>
+          <t>SOC 2 Type I (Vanta)</t>
+        </is>
+      </c>
+      <c r="B27" s="102" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="C27" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="F27" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" s="97">
+        <f>MIN(0.9, (C27*0.25 + D27*0.25 + E27*0.15 + F27*0.25 + G27*0.10)/5)</f>
+        <v/>
+      </c>
+      <c r="I27" s="98" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="J27" s="99">
+        <f>MAX(0.15, H27 + I27)</f>
+        <v/>
+      </c>
+      <c r="K27" s="21" t="inlineStr">
+        <is>
+          <t>Démarrage Next, certif Later</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Grilles de notation (0–5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>Facteur</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>D — Discovery</t>
+        </is>
+      </c>
+      <c r="B32" s="103" t="inlineStr">
+        <is>
+          <t>Hypothèse</t>
+        </is>
+      </c>
+      <c r="C32" s="103" t="inlineStr">
+        <is>
+          <t>1 entretien</t>
+        </is>
+      </c>
+      <c r="D32" s="103" t="inlineStr">
+        <is>
+          <t>2-3 entretiens</t>
+        </is>
+      </c>
+      <c r="E32" s="103" t="inlineStr">
+        <is>
+          <t>4+ entretiens, JTBD</t>
+        </is>
+      </c>
+      <c r="F32" s="103" t="inlineStr">
+        <is>
+          <t>Persona + data quanti</t>
+        </is>
+      </c>
+      <c r="G32" s="103" t="inlineStr">
+        <is>
+          <t>Pilote utilise / paie</t>
+        </is>
+      </c>
+      <c r="H32" s="47" t="n"/>
+      <c r="I32" s="47" t="n"/>
+      <c r="J32" s="47" t="n"/>
+      <c r="K32" s="47" t="n"/>
+    </row>
+    <row r="33" ht="36" customHeight="1">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>C — Capacity</t>
+        </is>
+      </c>
+      <c r="B33" s="103" t="inlineStr">
+        <is>
+          <t>Stack à choisir</t>
+        </is>
+      </c>
+      <c r="C33" s="103" t="inlineStr">
+        <is>
+          <t>Stack OK, 0 expert</t>
+        </is>
+      </c>
+      <c r="D33" s="103" t="inlineStr">
+        <is>
+          <t>Stack + spike OK</t>
+        </is>
+      </c>
+      <c r="E33" s="103" t="inlineStr">
+        <is>
+          <t>Similaire livré ailleurs</t>
+        </is>
+      </c>
+      <c r="F33" s="103" t="inlineStr">
+        <is>
+          <t>Identique livré ici</t>
+        </is>
+      </c>
+      <c r="G33" s="103" t="inlineStr">
+        <is>
+          <t>Code en place</t>
+        </is>
+      </c>
+      <c r="H33" s="47" t="n"/>
+      <c r="I33" s="47" t="n"/>
+      <c r="J33" s="47" t="n"/>
+      <c r="K33" s="47" t="n"/>
+    </row>
+    <row r="34" ht="36" customHeight="1">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>X — Dependencies</t>
+        </is>
+      </c>
+      <c r="B34" s="103" t="inlineStr">
+        <is>
+          <t>Bloqué (API fermée)</t>
+        </is>
+      </c>
+      <c r="C34" s="103" t="inlineStr">
+        <is>
+          <t>Négo incertaine</t>
+        </is>
+      </c>
+      <c r="D34" s="103" t="inlineStr">
+        <is>
+          <t>Plan B identifié</t>
+        </is>
+      </c>
+      <c r="E34" s="103" t="inlineStr">
+        <is>
+          <t>Contrat signé</t>
+        </is>
+      </c>
+      <c r="F34" s="103" t="inlineStr">
+        <is>
+          <t>0 dép. externe critique</t>
+        </is>
+      </c>
+      <c r="G34" s="103" t="inlineStr">
+        <is>
+          <t>Aucune dép. externe</t>
+        </is>
+      </c>
+      <c r="H34" s="47" t="n"/>
+      <c r="I34" s="47" t="n"/>
+      <c r="J34" s="47" t="n"/>
+      <c r="K34" s="47" t="n"/>
+    </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>M — Market</t>
+        </is>
+      </c>
+      <c r="B35" s="103" t="inlineStr">
+        <is>
+          <t>Pas de signal</t>
+        </is>
+      </c>
+      <c r="C35" s="103" t="inlineStr">
+        <is>
+          <t>1-2 demandes</t>
+        </is>
+      </c>
+      <c r="D35" s="103" t="inlineStr">
+        <is>
+          <t>5+ spontanées</t>
+        </is>
+      </c>
+      <c r="E35" s="103" t="inlineStr">
+        <is>
+          <t>10+ comptes docs</t>
+        </is>
+      </c>
+      <c r="F35" s="103" t="inlineStr">
+        <is>
+          <t>LOI / pré-commandes</t>
+        </is>
+      </c>
+      <c r="G35" s="103" t="inlineStr">
+        <is>
+          <t>Cohorte demande, upcharge</t>
+        </is>
+      </c>
+      <c r="H35" s="47" t="n"/>
+      <c r="I35" s="47" t="n"/>
+      <c r="J35" s="47" t="n"/>
+      <c r="K35" s="47" t="n"/>
+    </row>
+    <row r="36" ht="36" customHeight="1">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>R — Regulatory</t>
+        </is>
+      </c>
+      <c r="B36" s="103" t="inlineStr">
+        <is>
+          <t>Risque majeur inconnu</t>
+        </is>
+      </c>
+      <c r="C36" s="103" t="inlineStr">
+        <is>
+          <t>Cadre flou</t>
+        </is>
+      </c>
+      <c r="D36" s="103" t="inlineStr">
+        <is>
+          <t>Cadre + plan</t>
+        </is>
+      </c>
+      <c r="E36" s="103" t="inlineStr">
+        <is>
+          <t>Plan validé legal</t>
+        </is>
+      </c>
+      <c r="F36" s="103" t="inlineStr">
+        <is>
+          <t>Conforme + preuves</t>
+        </is>
+      </c>
+      <c r="G36" s="103" t="inlineStr">
+        <is>
+          <t>Certifié OACIQ/SOC2</t>
+        </is>
+      </c>
+      <c r="H36" s="47" t="n"/>
+      <c r="I36" s="47" t="n"/>
+      <c r="J36" s="47" t="n"/>
+      <c r="K36" s="47" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Notes méthode</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>1. Pondérations : D 25% · C 25% · X 15% · M 25% · R 10%. Sommé puis ramené sur 100%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>2. Plafond 90% (règle prr — aucun thème ne sort à 100%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>3. Plancher 15% (sous : appartient au backlog Discovery, pas à la roadmap).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>4. Discount = ajustement prudence négatif uniquement (jamais positif). Trois cas : petit n, externe, marché nouveau.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>5. Doc complète : klaris-confidence-methodology.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A30:K30"/>
+    <mergeCell ref="A39:K39"/>
+    <mergeCell ref="A43:K43"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A40:K40"/>
+  </mergeCells>
+  <conditionalFormatting sqref="J6:J27">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0.15"/>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="0.9"/>
+        <color rgb="00D64C2E"/>
+        <color rgb="00E0A836"/>
+        <color rgb="0050A04B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>